<commit_message>
Benutzerfreundlichkeit des Updateprozesses verbessert. Benutzeroberfläche vereinfacht. Excel Konflikt wird präventiv verhindert.
</commit_message>
<xml_diff>
--- a/Excel Template.xlsx
+++ b/Excel Template.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28730"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29929"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jonas\Documents\Repetierer\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\timow\Desktop\Projekte\Repetierer\Repetierer\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B9E0598-6457-4E5A-8DF2-8C8E54DF8443}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A441609-A193-4C07-8056-C24A578FA0E5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-93" yWindow="-93" windowWidth="20186" windowHeight="12800" tabRatio="500" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-93" yWindow="-93" windowWidth="25786" windowHeight="15466" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Class 1" sheetId="1" r:id="rId1"/>
@@ -38,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="111" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="91" uniqueCount="37">
   <si>
     <t>repetierer</t>
   </si>
@@ -502,404 +502,224 @@
       </c>
     </row>
     <row r="11" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A11" t="s">
-        <v>10</v>
-      </c>
       <c r="B11" s="1"/>
       <c r="C11" s="1"/>
       <c r="D11" s="1"/>
       <c r="E11" s="1"/>
       <c r="F11" s="1"/>
       <c r="G11" s="1"/>
-      <c r="I11" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J11" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
+      <c r="I11" s="1"/>
+      <c r="J11" s="1"/>
     </row>
     <row r="12" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A12" t="s">
-        <v>11</v>
-      </c>
       <c r="B12" s="1"/>
       <c r="C12" s="1"/>
       <c r="D12" s="1"/>
       <c r="E12" s="1"/>
       <c r="F12" s="1"/>
       <c r="G12" s="1"/>
-      <c r="I12" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J12" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
+      <c r="I12" s="1"/>
+      <c r="J12" s="1"/>
     </row>
     <row r="13" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A13" t="s">
-        <v>12</v>
-      </c>
       <c r="B13" s="1"/>
       <c r="C13" s="1"/>
       <c r="D13" s="1"/>
       <c r="E13" s="1"/>
       <c r="F13" s="1"/>
       <c r="G13" s="1"/>
-      <c r="I13" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J13" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
+      <c r="I13" s="1"/>
+      <c r="J13" s="1"/>
     </row>
     <row r="14" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A14" t="s">
-        <v>13</v>
-      </c>
       <c r="B14" s="1"/>
       <c r="C14" s="1"/>
       <c r="D14" s="1"/>
       <c r="E14" s="1"/>
       <c r="F14" s="1"/>
       <c r="G14" s="1"/>
-      <c r="I14" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J14" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
+      <c r="I14" s="1"/>
+      <c r="J14" s="1"/>
     </row>
     <row r="15" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A15" t="s">
-        <v>14</v>
-      </c>
       <c r="B15" s="1"/>
       <c r="C15" s="1"/>
       <c r="D15" s="1"/>
       <c r="E15" s="1"/>
       <c r="F15" s="1"/>
       <c r="G15" s="1"/>
-      <c r="I15" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J15" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
+      <c r="I15" s="1"/>
+      <c r="J15" s="1"/>
     </row>
     <row r="16" spans="1:17" ht="15" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A16" t="s">
-        <v>15</v>
-      </c>
       <c r="B16" s="1"/>
       <c r="C16" s="1"/>
       <c r="D16" s="1"/>
       <c r="E16" s="1"/>
       <c r="F16" s="1"/>
       <c r="G16" s="1"/>
-      <c r="I16" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J16" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="17" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A17" t="s">
-        <v>16</v>
-      </c>
+      <c r="I16" s="1"/>
+      <c r="J16" s="1"/>
+    </row>
+    <row r="17" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B17" s="1"/>
       <c r="C17" s="1"/>
       <c r="D17" s="1"/>
       <c r="E17" s="1"/>
       <c r="F17" s="1"/>
       <c r="G17" s="1"/>
-      <c r="I17" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J17" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="18" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A18" t="s">
-        <v>17</v>
-      </c>
+      <c r="I17" s="1"/>
+      <c r="J17" s="1"/>
+    </row>
+    <row r="18" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B18" s="1"/>
       <c r="C18" s="1"/>
       <c r="D18" s="1"/>
       <c r="E18" s="1"/>
       <c r="F18" s="1"/>
       <c r="G18" s="1"/>
-      <c r="I18" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J18" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="19" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A19" t="s">
-        <v>18</v>
-      </c>
+      <c r="I18" s="1"/>
+      <c r="J18" s="1"/>
+    </row>
+    <row r="19" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B19" s="1"/>
       <c r="C19" s="1"/>
       <c r="D19" s="1"/>
       <c r="E19" s="1"/>
       <c r="F19" s="1"/>
       <c r="G19" s="1"/>
-      <c r="I19" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J19" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="20" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A20" t="s">
-        <v>19</v>
-      </c>
+      <c r="I19" s="1"/>
+      <c r="J19" s="1"/>
+    </row>
+    <row r="20" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B20" s="1"/>
       <c r="C20" s="1"/>
       <c r="D20" s="1"/>
       <c r="E20" s="1"/>
       <c r="F20" s="1"/>
       <c r="G20" s="1"/>
-      <c r="I20" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J20" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="21" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A21" t="s">
-        <v>20</v>
-      </c>
+      <c r="I20" s="1"/>
+      <c r="J20" s="1"/>
+    </row>
+    <row r="21" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B21" s="1"/>
       <c r="C21" s="1"/>
       <c r="D21" s="1"/>
       <c r="E21" s="1"/>
       <c r="F21" s="1"/>
       <c r="G21" s="1"/>
-      <c r="I21" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J21" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="22" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A22" t="s">
-        <v>21</v>
-      </c>
+      <c r="I21" s="1"/>
+      <c r="J21" s="1"/>
+    </row>
+    <row r="22" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B22" s="1"/>
       <c r="C22" s="1"/>
       <c r="D22" s="1"/>
       <c r="E22" s="1"/>
       <c r="F22" s="1"/>
       <c r="G22" s="1"/>
-      <c r="I22" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J22" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="23" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A23" t="s">
-        <v>22</v>
-      </c>
+      <c r="I22" s="1"/>
+      <c r="J22" s="1"/>
+    </row>
+    <row r="23" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B23" s="1"/>
       <c r="C23" s="1"/>
       <c r="D23" s="1"/>
       <c r="E23" s="1"/>
       <c r="F23" s="1"/>
       <c r="G23" s="1"/>
-      <c r="I23" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J23" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="24" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A24" t="s">
-        <v>23</v>
-      </c>
+      <c r="I23" s="1"/>
+      <c r="J23" s="1"/>
+    </row>
+    <row r="24" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B24" s="1"/>
       <c r="C24" s="1"/>
       <c r="D24" s="1"/>
       <c r="E24" s="1"/>
       <c r="F24" s="1"/>
       <c r="G24" s="1"/>
-      <c r="I24" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J24" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="25" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A25" t="s">
-        <v>24</v>
-      </c>
+      <c r="I24" s="1"/>
+      <c r="J24" s="1"/>
+    </row>
+    <row r="25" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B25" s="1"/>
       <c r="C25" s="1"/>
       <c r="D25" s="1"/>
       <c r="E25" s="1"/>
       <c r="F25" s="1"/>
       <c r="G25" s="1"/>
-      <c r="I25" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J25" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="26" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A26" t="s">
-        <v>25</v>
-      </c>
+      <c r="I25" s="1"/>
+      <c r="J25" s="1"/>
+    </row>
+    <row r="26" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B26" s="1"/>
       <c r="C26" s="1"/>
       <c r="D26" s="1"/>
       <c r="E26" s="1"/>
       <c r="F26" s="1"/>
       <c r="G26" s="1"/>
-      <c r="I26" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J26" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="27" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A27" t="s">
-        <v>26</v>
-      </c>
+      <c r="I26" s="1"/>
+      <c r="J26" s="1"/>
+    </row>
+    <row r="27" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B27" s="1"/>
       <c r="C27" s="1"/>
       <c r="D27" s="1"/>
       <c r="E27" s="1"/>
       <c r="F27" s="1"/>
       <c r="G27" s="1"/>
-      <c r="I27" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J27" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="28" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A28" t="s">
-        <v>27</v>
-      </c>
+      <c r="I27" s="1"/>
+      <c r="J27" s="1"/>
+    </row>
+    <row r="28" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B28" s="1"/>
       <c r="C28" s="1"/>
       <c r="D28" s="1"/>
       <c r="E28" s="1"/>
       <c r="F28" s="1"/>
       <c r="G28" s="1"/>
-      <c r="I28" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J28" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="29" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A29" t="s">
-        <v>28</v>
-      </c>
+      <c r="I28" s="1"/>
+      <c r="J28" s="1"/>
+    </row>
+    <row r="29" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B29" s="1"/>
       <c r="C29" s="1"/>
       <c r="D29" s="1"/>
       <c r="E29" s="1"/>
       <c r="F29" s="1"/>
       <c r="G29" s="1"/>
-      <c r="I29" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J29" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
-    </row>
-    <row r="30" spans="1:10" ht="15" customHeight="1" x14ac:dyDescent="0.5">
-      <c r="A30" t="s">
-        <v>29</v>
-      </c>
+      <c r="I29" s="1"/>
+      <c r="J29" s="1"/>
+    </row>
+    <row r="30" spans="2:10" ht="15" customHeight="1" x14ac:dyDescent="0.5">
       <c r="B30" s="1"/>
       <c r="C30" s="1"/>
       <c r="D30" s="1"/>
       <c r="E30" s="1"/>
       <c r="F30" s="1"/>
       <c r="G30" s="1"/>
-      <c r="I30" s="1" t="str">
-        <f t="shared" si="0"/>
-        <v/>
-      </c>
-      <c r="J30" s="1" t="str">
-        <f t="shared" si="1"/>
-        <v/>
-      </c>
+      <c r="I30" s="1"/>
+      <c r="J30" s="1"/>
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="K3:K4"/>
+    <mergeCell ref="F3:F4"/>
+    <mergeCell ref="G3:G4"/>
+    <mergeCell ref="H3:H4"/>
+    <mergeCell ref="I3:I4"/>
+    <mergeCell ref="J3:J4"/>
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="C3:C4"/>
+    <mergeCell ref="D3:D4"/>
+    <mergeCell ref="E3:E4"/>
     <mergeCell ref="Q3:Q4"/>
     <mergeCell ref="L3:L4"/>
     <mergeCell ref="M3:M4"/>
     <mergeCell ref="N3:N4"/>
     <mergeCell ref="O3:O4"/>
     <mergeCell ref="P3:P4"/>
-    <mergeCell ref="A3:A4"/>
-    <mergeCell ref="B3:B4"/>
-    <mergeCell ref="C3:C4"/>
-    <mergeCell ref="D3:D4"/>
-    <mergeCell ref="E3:E4"/>
-    <mergeCell ref="K3:K4"/>
-    <mergeCell ref="F3:F4"/>
-    <mergeCell ref="G3:G4"/>
-    <mergeCell ref="H3:H4"/>
-    <mergeCell ref="I3:I4"/>
-    <mergeCell ref="J3:J4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78749999999999998" bottom="0.78749999999999998" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300"/>
@@ -1465,23 +1285,23 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="K3:K4"/>
+    <mergeCell ref="F3:F4"/>
+    <mergeCell ref="G3:G4"/>
+    <mergeCell ref="H3:H4"/>
+    <mergeCell ref="I3:I4"/>
+    <mergeCell ref="J3:J4"/>
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="C3:C4"/>
+    <mergeCell ref="D3:D4"/>
+    <mergeCell ref="E3:E4"/>
     <mergeCell ref="Q3:Q4"/>
     <mergeCell ref="L3:L4"/>
     <mergeCell ref="M3:M4"/>
     <mergeCell ref="N3:N4"/>
     <mergeCell ref="O3:O4"/>
     <mergeCell ref="P3:P4"/>
-    <mergeCell ref="A3:A4"/>
-    <mergeCell ref="B3:B4"/>
-    <mergeCell ref="C3:C4"/>
-    <mergeCell ref="D3:D4"/>
-    <mergeCell ref="E3:E4"/>
-    <mergeCell ref="K3:K4"/>
-    <mergeCell ref="F3:F4"/>
-    <mergeCell ref="G3:G4"/>
-    <mergeCell ref="H3:H4"/>
-    <mergeCell ref="I3:I4"/>
-    <mergeCell ref="J3:J4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78749999999999998" bottom="0.78749999999999998" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300"/>
@@ -2047,23 +1867,23 @@
     </row>
   </sheetData>
   <mergeCells count="17">
+    <mergeCell ref="K3:K4"/>
+    <mergeCell ref="F3:F4"/>
+    <mergeCell ref="G3:G4"/>
+    <mergeCell ref="H3:H4"/>
+    <mergeCell ref="I3:I4"/>
+    <mergeCell ref="J3:J4"/>
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="C3:C4"/>
+    <mergeCell ref="D3:D4"/>
+    <mergeCell ref="E3:E4"/>
     <mergeCell ref="Q3:Q4"/>
     <mergeCell ref="L3:L4"/>
     <mergeCell ref="M3:M4"/>
     <mergeCell ref="N3:N4"/>
     <mergeCell ref="O3:O4"/>
     <mergeCell ref="P3:P4"/>
-    <mergeCell ref="A3:A4"/>
-    <mergeCell ref="B3:B4"/>
-    <mergeCell ref="C3:C4"/>
-    <mergeCell ref="D3:D4"/>
-    <mergeCell ref="E3:E4"/>
-    <mergeCell ref="K3:K4"/>
-    <mergeCell ref="F3:F4"/>
-    <mergeCell ref="G3:G4"/>
-    <mergeCell ref="H3:H4"/>
-    <mergeCell ref="I3:I4"/>
-    <mergeCell ref="J3:J4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.78749999999999998" bottom="0.78749999999999998" header="0.511811023622047" footer="0.511811023622047"/>
   <pageSetup paperSize="9" orientation="portrait" useFirstPageNumber="1" horizontalDpi="300" verticalDpi="300"/>

</xml_diff>